<commit_message>
feat: Update SuperClaude v2.0.9 configurations and add new agents
- Add 40+ new specialized agents (ai-engineer, data-scientist, etc.)
- Update existing agent definitions and prompts
- Add new skills and commands
- Update rules for Python, Go, React, SQL trading
- Sync latest persona and documentation updates

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/modules/trading/reports/export/daily_history.xlsx
+++ b/modules/trading/reports/export/daily_history.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -623,6 +623,92 @@
       </c>
       <c r="M4" s="3" t="n">
         <v>0.71</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>17.01</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>60.73</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>5067.5</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>154.73</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>25859.25</v>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>6975.5</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>78409</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>4.24</v>
+      </c>
+      <c r="L5" s="3" t="n">
+        <v>3.53</v>
+      </c>
+      <c r="M5" s="3" t="n">
+        <v>0.74</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>18.52</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>59.2</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>4814.4</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>154.78</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>25486.75</v>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>6936.5</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>77773</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>3.68</v>
+      </c>
+      <c r="K6" s="3" t="n">
+        <v>4.24</v>
+      </c>
+      <c r="L6" s="3" t="n">
+        <v>3.53</v>
+      </c>
+      <c r="M6" s="3" t="n">
+        <v>0.74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>